<commit_message>
Fig 3: restore Sotalol Contractility overlay, tighten Vandetanib O2 filter, explicit axis reference
- generate_paper_figures.py: restore original _FIG3E_PANELS config (Sotalol 5.0/2.5/0.313 mM)
  and add upper/lower bounds to Vandetanib O2 outlier filter
- Regenerate Fig 3e O2 + Contractility PNGs, data Excel, and axisless variants
- Add 3 separate axisless Fig 3d scatter panels (Arrhythmia/HeartDamage/ConcernBinary)
- Add standalone Fig 3e legends (O2 + Contractility) in Axisless/
- Rewrite all Axis_Scaling_Reference.xlsx with explicit min/max/tick/step values
  (no 'auto' placeholders, categorical axes list actual category names, heatmap
  colorbar min/white/max added)
- Add Fig 4/5 axis reference sheets for 5x5 3D surface grids

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Output/PowerPoint_Figures/Fig_2/Axisless/Axis_Scaling_Reference.xlsx
+++ b/Output/PowerPoint_Figures/Fig_2/Axisless/Axis_Scaling_Reference.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fig_2_Axis_Info" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Fig_2_Axis_Info" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,34 +413,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X8"/>
+  <dimension ref="A1:AB8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="7" customWidth="1" min="2" max="2"/>
-    <col width="45" customWidth="1" min="3" max="3"/>
-    <col width="24" customWidth="1" min="4" max="4"/>
-    <col width="32" customWidth="1" min="5" max="5"/>
-    <col width="13" customWidth="1" min="6" max="6"/>
-    <col width="21" customWidth="1" min="7" max="7"/>
-    <col width="7" customWidth="1" min="8" max="8"/>
-    <col width="7" customWidth="1" min="9" max="9"/>
-    <col width="7" customWidth="1" min="10" max="10"/>
-    <col width="7" customWidth="1" min="11" max="11"/>
-    <col width="24" customWidth="1" min="12" max="12"/>
-    <col width="31" customWidth="1" min="13" max="13"/>
-    <col width="19" customWidth="1" min="14" max="14"/>
-    <col width="20" customWidth="1" min="15" max="15"/>
-    <col width="19" customWidth="1" min="16" max="16"/>
-    <col width="20" customWidth="1" min="17" max="17"/>
-    <col width="19" customWidth="1" min="18" max="18"/>
-    <col width="20" customWidth="1" min="19" max="19"/>
-    <col width="5" customWidth="1" min="20" max="20"/>
-    <col width="50" customWidth="1" min="21" max="21"/>
-    <col width="14" customWidth="1" min="22" max="22"/>
-    <col width="14" customWidth="1" min="23" max="23"/>
-    <col width="19" customWidth="1" min="24" max="24"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -505,62 +479,82 @@
       </c>
       <c r="M1" t="inlineStr">
         <is>
+          <t>X_Tick_Step</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
           <t>Y_Ticks</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>Y_Tick_Step</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>Colorbar_Min</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>Colorbar_White</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>Colorbar_Max</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>Colorbar_Label</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>Colorbar_Tick_Step</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
         <is>
           <t>Original_Width_in</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>Original_Height_in</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>Axisless_Width_in</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>Axisless_Height_in</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>Axisless_Width_px</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>Axisless_Height_px</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="AA1" t="inlineStr">
         <is>
           <t>DPI</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="AB1" t="inlineStr">
         <is>
           <t>Notes</t>
-        </is>
-      </c>
-      <c r="V1" t="inlineStr">
-        <is>
-          <t>Colorbar_Min</t>
-        </is>
-      </c>
-      <c r="W1" t="inlineStr">
-        <is>
-          <t>Colorbar_Max</t>
-        </is>
-      </c>
-      <c r="X1" t="inlineStr">
-        <is>
-          <t>Colorbar_Label</t>
         </is>
       </c>
     </row>
@@ -582,17 +576,17 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Drug</t>
+          <t>SNR Bucket Midpoint</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Count / SNR</t>
+          <t>Measurement Count</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>categorical</t>
+          <t>linear</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -600,63 +594,65 @@
           <t>linear</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
+      <c r="H2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="I2" t="n">
+        <v>10</v>
       </c>
       <c r="J2" t="n">
         <v>0</v>
       </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>auto</t>
-        </is>
+      <c r="K2" t="n">
+        <v>376347</v>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>drug names</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>auto</t>
-        </is>
-      </c>
-      <c r="N2" t="n">
+          <t>-1, 0, 1, 2, 3, 4, 5, 6, 7, 8, 9, 10</t>
+        </is>
+      </c>
+      <c r="M2" t="n">
+        <v>1</v>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>0, 50000, 100000, 150000, 200000, 250000, 300000, 350000, 400000</t>
+        </is>
+      </c>
+      <c r="O2" t="n">
+        <v>50000</v>
+      </c>
+      <c r="P2" t="inlineStr"/>
+      <c r="Q2" t="inlineStr"/>
+      <c r="R2" t="inlineStr"/>
+      <c r="S2" t="inlineStr"/>
+      <c r="T2" t="inlineStr"/>
+      <c r="U2" t="n">
         <v>9.890000000000001</v>
       </c>
-      <c r="O2" t="n">
+      <c r="V2" t="n">
         <v>5.89</v>
       </c>
-      <c r="P2" t="n">
+      <c r="W2" t="n">
         <v>9.140000000000001</v>
       </c>
-      <c r="Q2" t="n">
+      <c r="X2" t="n">
         <v>5.02</v>
       </c>
-      <c r="R2" t="n">
+      <c r="Y2" t="n">
         <v>5481</v>
       </c>
-      <c r="S2" t="n">
+      <c r="Z2" t="n">
         <v>3010</v>
       </c>
-      <c r="T2" t="n">
+      <c r="AA2" t="n">
         <v>600</v>
       </c>
-      <c r="U2" t="inlineStr">
-        <is>
-          <t>Stacked bar chart, SNR threshold line at 0.4</t>
-        </is>
-      </c>
-      <c r="V2" t="inlineStr"/>
-      <c r="W2" t="inlineStr"/>
-      <c r="X2" t="inlineStr"/>
+      <c r="AB2" t="inlineStr">
+        <is>
+          <t>Stacked bar: count per SNR bucket (101 buckets, 0.1 wide). Red threshold line at SNR=0.4.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -704,47 +700,55 @@
         <v>0</v>
       </c>
       <c r="K3" t="n">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="L3" t="inlineStr">
         <is>
           <t>0, 20, 40, 60, 80, 100</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr">
+      <c r="M3" t="n">
+        <v>20</v>
+      </c>
+      <c r="N3" t="inlineStr">
         <is>
           <t>0, 10, 20, 30, 40, 50, 60, 70</t>
         </is>
       </c>
-      <c r="N3" t="n">
+      <c r="O3" t="n">
+        <v>10</v>
+      </c>
+      <c r="P3" t="inlineStr"/>
+      <c r="Q3" t="inlineStr"/>
+      <c r="R3" t="inlineStr"/>
+      <c r="S3" t="inlineStr"/>
+      <c r="T3" t="inlineStr"/>
+      <c r="U3" t="n">
         <v>9.130000000000001</v>
       </c>
-      <c r="O3" t="n">
+      <c r="V3" t="n">
         <v>6.4</v>
       </c>
-      <c r="P3" t="n">
+      <c r="W3" t="n">
         <v>10.02</v>
       </c>
-      <c r="Q3" t="n">
+      <c r="X3" t="n">
         <v>7.02</v>
       </c>
-      <c r="R3" t="n">
+      <c r="Y3" t="n">
         <v>6010</v>
       </c>
-      <c r="S3" t="n">
+      <c r="Z3" t="n">
         <v>4210</v>
       </c>
-      <c r="T3" t="n">
+      <c r="AA3" t="n">
         <v>600</v>
       </c>
-      <c r="U3" t="inlineStr">
-        <is>
-          <t>Epirubicin O2 averaged dose-response, 8 concentrations</t>
-        </is>
-      </c>
-      <c r="V3" t="inlineStr"/>
-      <c r="W3" t="inlineStr"/>
-      <c r="X3" t="inlineStr"/>
+      <c r="AB3" t="inlineStr">
+        <is>
+          <t>Epirubicin O2 averaged, 9 concentrations (12/6/3/1.5/0.75/0.38/0.19/0.094 mM + offset-shifted edges)</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -801,38 +805,48 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
+          <t>x10 per decade</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
           <t>0, 20, 40, 60, 80, 100</t>
         </is>
       </c>
-      <c r="N4" t="n">
+      <c r="O4" t="n">
+        <v>20</v>
+      </c>
+      <c r="P4" t="inlineStr"/>
+      <c r="Q4" t="inlineStr"/>
+      <c r="R4" t="inlineStr"/>
+      <c r="S4" t="inlineStr"/>
+      <c r="T4" t="inlineStr"/>
+      <c r="U4" t="n">
         <v>3.8</v>
       </c>
-      <c r="O4" t="n">
+      <c r="V4" t="n">
         <v>2.59</v>
       </c>
-      <c r="P4" t="n">
+      <c r="W4" t="n">
         <v>3.19</v>
       </c>
-      <c r="Q4" t="n">
+      <c r="X4" t="n">
         <v>2.1</v>
       </c>
-      <c r="R4" t="n">
+      <c r="Y4" t="n">
         <v>1912</v>
       </c>
-      <c r="S4" t="n">
+      <c r="Z4" t="n">
         <v>1262</v>
       </c>
-      <c r="T4" t="n">
+      <c r="AA4" t="n">
         <v>600</v>
       </c>
-      <c r="U4" t="inlineStr">
-        <is>
-          <t>TC50=0.453 mM at 40h, 4PL sigmoid, wells excluded: {0,2,3,4,10,11,13,15}</t>
-        </is>
-      </c>
-      <c r="V4" t="inlineStr"/>
-      <c r="W4" t="inlineStr"/>
-      <c r="X4" t="inlineStr"/>
+      <c r="AB4" t="inlineStr">
+        <is>
+          <t>TC50=0.453 mM at 40h. 4PL sigmoid, wells excluded: {0,2,3,4,10,11,13,15}, 6 mM row dropped.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -857,7 +871,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Epirubicin Dose (sorted wells)</t>
+          <t>Epirubicin Dose (mM, grouped by conc)</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -867,7 +881,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>categorical (wells)</t>
+          <t>categorical (wells sorted within conc)</t>
         </is>
       </c>
       <c r="H5" t="n">
@@ -878,59 +892,71 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>(row 0 = top conc)</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>(row N = bottom)</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>time points</t>
-        </is>
-      </c>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>well labels</t>
-        </is>
-      </c>
-      <c r="N5" t="n">
-        <v>12.08</v>
-      </c>
-      <c r="O5" t="n">
-        <v>6.54</v>
+          <t>time-point subset (~every 10th label displayed)</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr"/>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>12, 6, 3, 1.5, 1, 0.75, 0.38, 0.19, 0.094  (19 wells total after dropping 0.38.1)</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>categorical (non-uniform bins)</t>
+        </is>
       </c>
       <c r="P5" t="n">
-        <v>9.56</v>
+        <v>0</v>
       </c>
       <c r="Q5" t="n">
-        <v>5.63</v>
+        <v>50</v>
       </c>
       <c r="R5" t="n">
-        <v>5733</v>
-      </c>
-      <c r="S5" t="n">
-        <v>3378</v>
+        <v>100</v>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>Oxygen (% Air) — actual data range 0 to 79.15 (never reaches pure red)</t>
+        </is>
       </c>
       <c r="T5" t="n">
+        <v>20</v>
+      </c>
+      <c r="U5" t="n">
+        <v>13.27</v>
+      </c>
+      <c r="V5" t="n">
+        <v>6.75</v>
+      </c>
+      <c r="W5" t="n">
+        <v>10.28</v>
+      </c>
+      <c r="X5" t="n">
+        <v>5.78</v>
+      </c>
+      <c r="Y5" t="n">
+        <v>6170</v>
+      </c>
+      <c r="Z5" t="n">
+        <v>3467</v>
+      </c>
+      <c r="AA5" t="n">
         <v>600</v>
       </c>
-      <c r="U5" t="inlineStr">
-        <is>
-          <t>LOWESS w=16, sorted wells, blue-white-red colormap</t>
-        </is>
-      </c>
-      <c r="V5" t="n">
-        <v>0</v>
-      </c>
-      <c r="W5" t="n">
-        <v>100</v>
-      </c>
-      <c r="X5" t="inlineStr">
-        <is>
-          <t>Oxygen (% Air)</t>
+      <c r="AB5" t="inlineStr">
+        <is>
+          <t>LOWESS w=16, sorted wells ascending within conc. Colormap: #123BFF -&gt; white -&gt; #FF2908.</t>
         </is>
       </c>
     </row>
@@ -976,55 +1002,59 @@
       <c r="I6" t="n">
         <v>100</v>
       </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>auto</t>
-        </is>
-      </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>auto</t>
-        </is>
+      <c r="J6" t="n">
+        <v>2.73</v>
+      </c>
+      <c r="K6" t="n">
+        <v>11.12</v>
       </c>
       <c r="L6" t="inlineStr">
         <is>
           <t>0, 20, 40, 60, 80, 100</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr">
-        <is>
-          <t>auto</t>
-        </is>
-      </c>
-      <c r="N6" t="n">
-        <v>10.84</v>
+      <c r="M6" t="n">
+        <v>20</v>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>3, 4, 5, 6, 7, 8, 9, 10, 11  (matplotlib auto on [2.73, 11.12])</t>
+        </is>
       </c>
       <c r="O6" t="n">
-        <v>7.27</v>
-      </c>
-      <c r="P6" t="n">
-        <v>12.02</v>
-      </c>
-      <c r="Q6" t="n">
-        <v>8.02</v>
-      </c>
-      <c r="R6" t="n">
-        <v>7210</v>
-      </c>
-      <c r="S6" t="n">
-        <v>4810</v>
-      </c>
-      <c r="T6" t="n">
+        <v>1</v>
+      </c>
+      <c r="P6" t="inlineStr"/>
+      <c r="Q6" t="inlineStr"/>
+      <c r="R6" t="inlineStr"/>
+      <c r="S6" t="inlineStr"/>
+      <c r="T6" t="inlineStr"/>
+      <c r="U6" t="n">
+        <v>9.890000000000001</v>
+      </c>
+      <c r="V6" t="n">
+        <v>7.82</v>
+      </c>
+      <c r="W6" t="n">
+        <v>10.02</v>
+      </c>
+      <c r="X6" t="n">
+        <v>7.02</v>
+      </c>
+      <c r="Y6" t="n">
+        <v>6010</v>
+      </c>
+      <c r="Z6" t="n">
+        <v>4210</v>
+      </c>
+      <c r="AA6" t="n">
         <v>600</v>
       </c>
-      <c r="U6" t="inlineStr">
-        <is>
-          <t>Mexiletine contractility averaged, 7 concentrations, offset to global avg start</t>
-        </is>
-      </c>
-      <c r="V6" t="inlineStr"/>
-      <c r="W6" t="inlineStr"/>
-      <c r="X6" t="inlineStr"/>
+      <c r="AB6" t="inlineStr">
+        <is>
+          <t>Mexiletine contractility averaged, 7 concs (20/10/5/2.5/1.25/0.625/0.156 mM). Shifted to global-avg start.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1049,7 +1079,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Contractility</t>
+          <t>Contractility (stacked offsets, arbitrary units)</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -1059,7 +1089,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>linear (stacked)</t>
+          <t>linear (stacked with vertical offset per dose)</t>
         </is>
       </c>
       <c r="H7" t="n">
@@ -1070,12 +1100,12 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>-0.5 * spacing</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>2.8 * spacing (spacing = 1.5 * max_ptp)</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
@@ -1083,40 +1113,50 @@
           <t>0, 1, 2, 3, 4, 5, 6, 7</t>
         </is>
       </c>
-      <c r="M7" t="inlineStr">
-        <is>
-          <t>none (stacked traces)</t>
-        </is>
-      </c>
-      <c r="N7" t="n">
-        <v>8.4</v>
-      </c>
-      <c r="O7" t="n">
-        <v>4.42</v>
-      </c>
-      <c r="P7" t="n">
+      <c r="M7" t="n">
+        <v>1</v>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>none (y-axis ticks hidden; traces stacked)</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>no ticks</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr"/>
+      <c r="Q7" t="inlineStr"/>
+      <c r="R7" t="inlineStr"/>
+      <c r="S7" t="inlineStr"/>
+      <c r="T7" t="inlineStr"/>
+      <c r="U7" t="n">
+        <v>9.890000000000001</v>
+      </c>
+      <c r="V7" t="n">
+        <v>8</v>
+      </c>
+      <c r="W7" t="n">
         <v>10.02</v>
       </c>
-      <c r="Q7" t="n">
-        <v>4.52</v>
-      </c>
-      <c r="R7" t="n">
+      <c r="X7" t="n">
+        <v>8</v>
+      </c>
+      <c r="Y7" t="n">
         <v>6010</v>
       </c>
-      <c r="S7" t="n">
-        <v>2710</v>
-      </c>
-      <c r="T7" t="n">
+      <c r="Z7" t="n">
+        <v>4800</v>
+      </c>
+      <c r="AA7" t="n">
         <v>600</v>
       </c>
-      <c r="U7" t="inlineStr">
-        <is>
-          <t>3 doses (5.0, 2.5, 0.625 mM) at 48h, CubicSpline smoothed</t>
-        </is>
-      </c>
-      <c r="V7" t="inlineStr"/>
-      <c r="W7" t="inlineStr"/>
-      <c r="X7" t="inlineStr"/>
+      <c r="AB7" t="inlineStr">
+        <is>
+          <t>3 doses stacked: Low=0.625 mM (plasma #fdb42f), Med=2.5 mM (plasma #cc4778), High=5.0 mM (plasma #9c179e). CubicSpline smoothed.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1141,7 +1181,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Mexiletine Dose (sorted wells)</t>
+          <t>Mexiletine Dose (mM, grouped by conc)</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -1151,7 +1191,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>categorical (wells)</t>
+          <t>categorical (wells sorted within conc)</t>
         </is>
       </c>
       <c r="H8" t="n">
@@ -1162,61 +1202,71 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>(row 0 = top conc)</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>(row N = bottom)</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>time points</t>
-        </is>
-      </c>
-      <c r="M8" t="inlineStr">
-        <is>
-          <t>well labels</t>
-        </is>
-      </c>
-      <c r="N8" t="n">
-        <v>11.31</v>
-      </c>
-      <c r="O8" t="n">
-        <v>5.82</v>
+          <t>time-point subset (~every 10th label displayed)</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr"/>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>20, 10, 5, 2.5, 1.25, 0.625, 0.156  (14 wells after exclusions)</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>categorical (non-uniform bins)</t>
+        </is>
       </c>
       <c r="P8" t="n">
-        <v>8.970000000000001</v>
+        <v>0</v>
       </c>
       <c r="Q8" t="n">
-        <v>4.91</v>
+        <v>12.28</v>
       </c>
       <c r="R8" t="n">
-        <v>5379</v>
-      </c>
-      <c r="S8" t="n">
-        <v>2946</v>
+        <v>24.56</v>
+      </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>Contractility (%) — vmin=0, vmax=auto=24.56 (white at midpoint 12.28)</t>
+        </is>
       </c>
       <c r="T8" t="n">
+        <v>4.912</v>
+      </c>
+      <c r="U8" t="n">
+        <v>13.27</v>
+      </c>
+      <c r="V8" t="n">
+        <v>6.75</v>
+      </c>
+      <c r="W8" t="n">
+        <v>10.28</v>
+      </c>
+      <c r="X8" t="n">
+        <v>5.78</v>
+      </c>
+      <c r="Y8" t="n">
+        <v>6170</v>
+      </c>
+      <c r="Z8" t="n">
+        <v>3467</v>
+      </c>
+      <c r="AA8" t="n">
         <v>600</v>
       </c>
-      <c r="U8" t="inlineStr">
-        <is>
-          <t>LOWESS w=16, sorted wells, blue-white-red colormap</t>
-        </is>
-      </c>
-      <c r="V8" t="n">
-        <v>0</v>
-      </c>
-      <c r="W8" t="inlineStr">
-        <is>
-          <t>auto</t>
-        </is>
-      </c>
-      <c r="X8" t="inlineStr">
-        <is>
-          <t>Contractility (%)</t>
+      <c r="AB8" t="inlineStr">
+        <is>
+          <t>LOWESS w=16, sorted ascending. Colormap: #123BFF -&gt; white -&gt; #FF2908. vmax auto = data max.</t>
         </is>
       </c>
     </row>

</xml_diff>